<commit_message>
Batch 19 shipped: the no-input parts (+76 OMi parts, 1,607 of 2,535)
- answered rows (A1/A8/A10/A11/A12/A18), own-STEP rows, Brennan cells (Q1)
- new masters 0319 2500 2603 2613 3474 6603 FS2500N1; 2500HX/2603HX retired (A7)
- 2502 parked (QA #180); rows needing the user listed in QA #181
- dry runs 31/31 PASS, post-ship verify 0 BAD; QA_Log #179-#181, coverage, status docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04_DESIGN_TABLES/DesignTable_0319.xlsx
+++ b/04_DESIGN_TABLES/DesignTable_0319.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>D@BORE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -504,7 +509,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 42 "Side 1 ID" 0.130 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -516,6 +521,9 @@
         <is>
           <t>0319-02</t>
         </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="4">
@@ -547,7 +555,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 43 "Side 1 ID" 0.193 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -559,6 +567,9 @@
         <is>
           <t>0319-03</t>
         </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="5">
@@ -590,7 +601,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 44 "Side 1 ID" 0.255 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -602,6 +613,9 @@
         <is>
           <t>0319-04</t>
         </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0.255</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +647,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 45 "Side 1 ID" 0.318 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -645,6 +659,9 @@
         <is>
           <t>0319-05</t>
         </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0.318</v>
       </c>
     </row>
     <row r="7">
@@ -676,7 +693,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 46 "Side 1 ID" 0.380 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -688,6 +705,9 @@
         <is>
           <t>0319-06</t>
         </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0.38</v>
       </c>
     </row>
     <row r="8">
@@ -719,7 +739,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 47 "Side 1 ID" 0.505 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -731,6 +751,9 @@
         <is>
           <t>0319-08</t>
         </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0.505</v>
       </c>
     </row>
     <row r="9">
@@ -762,7 +785,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 48 "Side 1 ID" 0.631 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -774,6 +797,9 @@
         <is>
           <t>0319-10</t>
         </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0.631</v>
       </c>
     </row>
     <row r="10">
@@ -805,7 +831,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 49 "Side 1 ID" 0.756 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -817,6 +843,9 @@
         <is>
           <t>0319-12</t>
         </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.756</v>
       </c>
     </row>
     <row r="11">
@@ -891,7 +920,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 50 "Side 1 ID" 1.006 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -903,6 +932,9 @@
         <is>
           <t>0319-16</t>
         </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1.006</v>
       </c>
     </row>
     <row r="13">
@@ -934,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 51 "Side 1 ID" 1.260 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -946,6 +978,9 @@
         <is>
           <t>0319-20</t>
         </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1.26</v>
       </c>
     </row>
     <row r="14">
@@ -977,7 +1012,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 52 "Side 1 ID" 1.510 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -989,6 +1024,9 @@
         <is>
           <t>0319-24</t>
         </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1.51</v>
       </c>
     </row>
     <row r="15">
@@ -1020,7 +1058,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed)</t>
+          <t>Air-Way s48 only (double-pass 13 rows); Air-Way part numbers printed as 319-n; config names zero-padded to 0319-nn; sleeve has no thread column (X = sleeve OD as printed) | bore D@BORE: OMi WebsitePartsInfo2026 Items row 53 "Side 1 ID" 2.014 (Air-Way s48 has no bore column; 2026-10-20, user A2)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1032,6 +1070,9 @@
         <is>
           <t>0319-32</t>
         </is>
+      </c>
+      <c r="L15" t="n">
+        <v>2.014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>